<commit_message>
changed file to excel
</commit_message>
<xml_diff>
--- a/Nike_Sales_Date_Cleaned.csv.xlsx
+++ b/Nike_Sales_Date_Cleaned.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\DATASCIENCE\project\Economy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{55B70D8D-AB55-416A-A81B-D4945E04EBC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F397D30B-A2D9-4963-97B5-2711590CFD09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{1BBA80CF-F85E-41DC-B451-552787AFA58E}"/>
   </bookViews>
@@ -668,9 +668,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1165,7 +1168,7 @@
       <c r="I4">
         <v>0</v>
       </c>
-      <c r="J4" s="1">
+      <c r="J4" s="2">
         <v>45392</v>
       </c>
       <c r="K4" t="s">

</xml_diff>